<commit_message>
Drop helm part2 - writing a chart (#122)
* drop exercise on helm chart writing
* update helm references
</commit_message>
<xml_diff>
--- a/admin/Agenda_4days_cleaned.xlsx
+++ b/admin/Agenda_4days_cleaned.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10908"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/d051945/SAPDevelop/git-repos/docker-k8s-training/admin/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/D051945/SAPDevelop/git-repos/docker-k8s-training/admin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4482CA29-D06B-5546-8E72-EFFBEC5A1883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE18159-09C4-F44D-8F37-96CA7B20BE60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="47220" yWindow="-2780" windowWidth="34640" windowHeight="21900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48860" yWindow="-3920" windowWidth="34640" windowHeight="21900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Day1" sheetId="29" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="97">
   <si>
     <t>Meeting Information:</t>
   </si>
@@ -345,9 +345,6 @@
     <t>Presentation: Gardener</t>
   </si>
   <si>
-    <t>Presentation: Helm</t>
-  </si>
-  <si>
     <t>12_helm.pptx</t>
   </si>
   <si>
@@ -357,12 +354,6 @@
     <t>Exercise: Helm Basics</t>
   </si>
   <si>
-    <t>(optional) Exercise: Writing A Helm Chart</t>
-  </si>
-  <si>
-    <t>exercise_11_write_a_helm_chart.md</t>
-  </si>
-  <si>
     <t>Presentation: Introducing the Fortune Cookies App</t>
   </si>
   <si>
@@ -379,6 +370,18 @@
   </si>
   <si>
     <t>Ask for feedback in the call (in case anyone wants to give some)</t>
+  </si>
+  <si>
+    <t>Presentation Jobs, CRDs, …</t>
+  </si>
+  <si>
+    <t>11_3_morePods_Scheduling.pptx</t>
+  </si>
+  <si>
+    <t>Presentation Helm</t>
+  </si>
+  <si>
+    <t>Exercise: Fortune Cookies with Breaks as you see fit</t>
   </si>
 </sst>
 </file>
@@ -686,7 +689,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -752,6 +755,21 @@
       <alignment textRotation="255" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="4" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -767,14 +785,9 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1168,10 +1181,10 @@
       <c r="M1" s="7"/>
     </row>
     <row r="2" spans="2:20" ht="0.5" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
       <c r="J2" s="19"/>
       <c r="K2" s="19" t="s">
         <v>1</v>
@@ -1182,10 +1195,10 @@
       <c r="M2" s="19"/>
     </row>
     <row r="3" spans="2:20" ht="0.5" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3">
         <v>0.375</v>
@@ -1289,14 +1302,14 @@
       <c r="E12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="33"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="38"/>
       <c r="L12" s="22" t="s">
         <v>6</v>
       </c>
@@ -1324,13 +1337,13 @@
         <f t="shared" ref="F13:F23" ca="1" si="2">ROW()-ROW(OFFSET(F13,-1,))+IF(ISERROR(OFFSET(F13,-1,)*1),0,OFFSET(F13,-1,))</f>
         <v>1</v>
       </c>
-      <c r="G13" s="34" t="s">
+      <c r="G13" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="36"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="33"/>
       <c r="L13" s="18" t="s">
         <v>11</v>
       </c>
@@ -1363,13 +1376,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F14,-1,))+IF(ISERROR(OFFSET(F14,-1,)*1),0,OFFSET(F14,-1,))</f>
         <v>2</v>
       </c>
-      <c r="G14" s="34" t="s">
+      <c r="G14" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="36"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="33"/>
       <c r="L14" s="18"/>
       <c r="M14" s="12" t="s">
         <v>23</v>
@@ -1402,13 +1415,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>3</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="36"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="33"/>
       <c r="L15" s="18"/>
       <c r="M15" s="12"/>
       <c r="N15" s="24"/>
@@ -1439,13 +1452,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>4</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="36"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
       <c r="L16" s="18"/>
       <c r="M16" s="12" t="s">
         <v>22</v>
@@ -1478,13 +1491,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F17,-1,))+IF(ISERROR(OFFSET(F17,-1,)*1),0,OFFSET(F17,-1,))</f>
         <v>5</v>
       </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="36"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="33"/>
       <c r="L17" s="18"/>
       <c r="M17" s="12" t="s">
         <v>25</v>
@@ -1517,13 +1530,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>6</v>
       </c>
-      <c r="G18" s="34" t="s">
+      <c r="G18" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="36"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="33"/>
       <c r="L18" s="18"/>
       <c r="M18" s="12"/>
       <c r="N18" s="26"/>
@@ -1554,13 +1567,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F19,-1,))+IF(ISERROR(OFFSET(F19,-1,)*1),0,OFFSET(F19,-1,))</f>
         <v>7</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="36"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="33"/>
       <c r="L19" s="18"/>
       <c r="M19" s="12" t="s">
         <v>28</v>
@@ -1593,13 +1606,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>8</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="G20" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="36"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="33"/>
       <c r="L20" s="18"/>
       <c r="M20" s="12" t="s">
         <v>31</v>
@@ -1632,13 +1645,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>9</v>
       </c>
-      <c r="G21" s="34" t="s">
+      <c r="G21" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="36"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="33"/>
       <c r="L21" s="18"/>
       <c r="M21" s="12" t="s">
         <v>32</v>
@@ -1671,13 +1684,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>10</v>
       </c>
-      <c r="G22" s="34" t="s">
+      <c r="G22" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="36"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="33"/>
       <c r="L22" s="18"/>
       <c r="M22" s="12" t="s">
         <v>28</v>
@@ -1710,13 +1723,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>11</v>
       </c>
-      <c r="G23" s="34" t="s">
+      <c r="G23" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="36"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="33"/>
       <c r="L23" s="18"/>
       <c r="M23" s="12"/>
       <c r="N23" s="26"/>
@@ -1747,13 +1760,13 @@
         <f t="shared" ref="F24:F26" ca="1" si="4">ROW()-ROW(OFFSET(F24,-1,))+IF(ISERROR(OFFSET(F24,-1,)*1),0,OFFSET(F24,-1,))</f>
         <v>12</v>
       </c>
-      <c r="G24" s="34" t="s">
+      <c r="G24" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="36"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="33"/>
       <c r="L24" s="18"/>
       <c r="M24" s="12" t="s">
         <v>35</v>
@@ -1786,13 +1799,13 @@
         <f t="shared" ca="1" si="4"/>
         <v>13</v>
       </c>
-      <c r="G25" s="34" t="s">
+      <c r="G25" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="35"/>
-      <c r="K25" s="36"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="33"/>
       <c r="L25" s="18"/>
       <c r="M25" s="12" t="s">
         <v>37</v>
@@ -1825,13 +1838,13 @@
         <f t="shared" ca="1" si="4"/>
         <v>14</v>
       </c>
-      <c r="G26" s="34" t="s">
+      <c r="G26" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35"/>
-      <c r="K26" s="36"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="33"/>
       <c r="L26" s="18"/>
       <c r="M26" s="12"/>
       <c r="N26" s="27"/>
@@ -1864,13 +1877,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="G20:K20"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G22:K22"/>
-    <mergeCell ref="G24:K24"/>
     <mergeCell ref="F2:I2"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="F12:K12"/>
@@ -1881,6 +1887,13 @@
     <mergeCell ref="G18:K18"/>
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="G16:K16"/>
+    <mergeCell ref="G20:K20"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G21:K21"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G22:K22"/>
+    <mergeCell ref="G24:K24"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="E27">
@@ -1933,10 +1946,10 @@
       <c r="M1" s="7"/>
     </row>
     <row r="2" spans="2:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
       <c r="J2" s="19"/>
       <c r="K2" s="19" t="s">
         <v>1</v>
@@ -1947,10 +1960,10 @@
       <c r="M2" s="19"/>
     </row>
     <row r="3" spans="2:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3">
         <v>0.375</v>
@@ -2054,14 +2067,14 @@
       <c r="E12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="33"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="38"/>
       <c r="L12" s="22" t="s">
         <v>6</v>
       </c>
@@ -2089,13 +2102,13 @@
         <f t="shared" ref="F13:F25" ca="1" si="2">ROW()-ROW(OFFSET(F13,-1,))+IF(ISERROR(OFFSET(F13,-1,)*1),0,OFFSET(F13,-1,))</f>
         <v>1</v>
       </c>
-      <c r="G13" s="34" t="s">
+      <c r="G13" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="36"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="33"/>
       <c r="L13" s="18"/>
       <c r="M13" s="12"/>
       <c r="N13" s="24"/>
@@ -2126,13 +2139,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F14,-1,))+IF(ISERROR(OFFSET(F14,-1,)*1),0,OFFSET(F14,-1,))</f>
         <v>2</v>
       </c>
-      <c r="G14" s="34" t="s">
+      <c r="G14" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="36"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="33"/>
       <c r="L14" s="18"/>
       <c r="M14" s="12" t="s">
         <v>40</v>
@@ -2165,13 +2178,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F15,-1,))+IF(ISERROR(OFFSET(F15,-1,)*1),0,OFFSET(F15,-1,))</f>
         <v>3</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="36"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="33"/>
       <c r="L15" s="18"/>
       <c r="M15" s="12" t="s">
         <v>42</v>
@@ -2204,13 +2217,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F16,-1,))+IF(ISERROR(OFFSET(F16,-1,)*1),0,OFFSET(F16,-1,))</f>
         <v>4</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="36"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
       <c r="L16" s="18"/>
       <c r="M16" s="12"/>
       <c r="N16" s="17"/>
@@ -2241,13 +2254,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>5</v>
       </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="36"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="33"/>
       <c r="L17" s="18"/>
       <c r="M17" s="12"/>
       <c r="N17" s="26"/>
@@ -2278,13 +2291,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>6</v>
       </c>
-      <c r="G18" s="34" t="s">
+      <c r="G18" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="36"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="33"/>
       <c r="L18" s="18"/>
       <c r="M18" s="12" t="s">
         <v>45</v>
@@ -2317,13 +2330,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>7</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="36"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="33"/>
       <c r="L19" s="18"/>
       <c r="M19" s="12" t="s">
         <v>47</v>
@@ -2356,13 +2369,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F20,-1,))+IF(ISERROR(OFFSET(F20,-1,)*1),0,OFFSET(F20,-1,))</f>
         <v>8</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="G20" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="36"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="33"/>
       <c r="L20" s="18"/>
       <c r="M20" s="12"/>
       <c r="N20" s="28"/>
@@ -2393,13 +2406,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>9</v>
       </c>
-      <c r="G21" s="34" t="s">
+      <c r="G21" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="36"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="33"/>
       <c r="L21" s="18"/>
       <c r="M21" s="12" t="s">
         <v>49</v>
@@ -2432,13 +2445,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>10</v>
       </c>
-      <c r="G22" s="34" t="s">
+      <c r="G22" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="36"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="33"/>
       <c r="L22" s="18"/>
       <c r="M22" s="12" t="s">
         <v>51</v>
@@ -2471,13 +2484,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>11</v>
       </c>
-      <c r="G23" s="34" t="s">
+      <c r="G23" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="36"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="33"/>
       <c r="L23" s="18"/>
       <c r="M23" s="12" t="s">
         <v>53</v>
@@ -2510,13 +2523,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>12</v>
       </c>
-      <c r="G24" s="34" t="s">
+      <c r="G24" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="36"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="33"/>
       <c r="L24" s="18"/>
       <c r="M24" s="12"/>
       <c r="N24" s="27"/>
@@ -2547,13 +2560,13 @@
         <f t="shared" ca="1" si="2"/>
         <v>13</v>
       </c>
-      <c r="G25" s="34" t="s">
+      <c r="G25" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="35"/>
-      <c r="K25" s="36"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="33"/>
       <c r="L25" s="18"/>
       <c r="M25" s="12" t="s">
         <v>55</v>
@@ -2586,13 +2599,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F26,-1,))+IF(ISERROR(OFFSET(F26,-1,)*1),0,OFFSET(F26,-1,))</f>
         <v>14</v>
       </c>
-      <c r="G26" s="34" t="s">
+      <c r="G26" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35"/>
-      <c r="K26" s="36"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="33"/>
       <c r="L26" s="18"/>
       <c r="M26" s="12" t="s">
         <v>57</v>
@@ -2625,13 +2638,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F27,-1,))+IF(ISERROR(OFFSET(F27,-1,)*1),0,OFFSET(F27,-1,))</f>
         <v>15</v>
       </c>
-      <c r="G27" s="34" t="s">
+      <c r="G27" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="35"/>
-      <c r="K27" s="36"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="33"/>
       <c r="L27" s="18"/>
       <c r="M27" s="12" t="s">
         <v>59</v>
@@ -2664,13 +2677,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F28,-1,))+IF(ISERROR(OFFSET(F28,-1,)*1),0,OFFSET(F28,-1,))</f>
         <v>16</v>
       </c>
-      <c r="G28" s="34" t="s">
+      <c r="G28" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="H28" s="35"/>
-      <c r="I28" s="35"/>
-      <c r="J28" s="35"/>
-      <c r="K28" s="36"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="33"/>
       <c r="L28" s="18"/>
       <c r="M28" s="12" t="s">
         <v>60</v>
@@ -2703,13 +2716,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F29,-1,))+IF(ISERROR(OFFSET(F29,-1,)*1),0,OFFSET(F29,-1,))</f>
         <v>17</v>
       </c>
-      <c r="G29" s="34" t="s">
+      <c r="G29" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35"/>
-      <c r="K29" s="36"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="33"/>
       <c r="L29" s="18"/>
       <c r="M29" s="12"/>
       <c r="N29" s="27"/>
@@ -2742,11 +2755,7 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="G25:K25"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G15:K15"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G28:K28"/>
+    <mergeCell ref="G29:K29"/>
     <mergeCell ref="F2:I2"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="F12:K12"/>
@@ -2761,7 +2770,11 @@
     <mergeCell ref="G21:K21"/>
     <mergeCell ref="G22:K22"/>
     <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G29:K29"/>
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G15:K15"/>
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G28:K28"/>
   </mergeCells>
   <conditionalFormatting sqref="E30">
     <cfRule type="expression" dxfId="2" priority="3" stopIfTrue="1">
@@ -2813,10 +2826,10 @@
       <c r="M1" s="7"/>
     </row>
     <row r="2" spans="2:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
       <c r="J2" s="19"/>
       <c r="K2" s="19" t="s">
         <v>1</v>
@@ -2827,10 +2840,10 @@
       <c r="M2" s="19"/>
     </row>
     <row r="3" spans="2:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3">
         <v>0.375</v>
@@ -2934,14 +2947,14 @@
       <c r="E12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="33"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="38"/>
       <c r="L12" s="22" t="s">
         <v>6</v>
       </c>
@@ -2969,13 +2982,13 @@
         <f t="shared" ref="F13:F26" ca="1" si="3">ROW()-ROW(OFFSET(F13,-1,))+IF(ISERROR(OFFSET(F13,-1,)*1),0,OFFSET(F13,-1,))</f>
         <v>1</v>
       </c>
-      <c r="G13" s="34" t="s">
+      <c r="G13" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="36"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="33"/>
       <c r="L13" s="18"/>
       <c r="M13" s="12"/>
       <c r="N13" s="24"/>
@@ -3006,13 +3019,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F14,-1,))+IF(ISERROR(OFFSET(F14,-1,)*1),0,OFFSET(F14,-1,))</f>
         <v>2</v>
       </c>
-      <c r="G14" s="34" t="s">
+      <c r="G14" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="36"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="33"/>
       <c r="L14" s="18"/>
       <c r="M14" s="12" t="s">
         <v>64</v>
@@ -3045,13 +3058,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>3</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="36"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="33"/>
       <c r="L15" s="18"/>
       <c r="M15" s="12" t="s">
         <v>66</v>
@@ -3084,13 +3097,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F16,-1,))+IF(ISERROR(OFFSET(F16,-1,)*1),0,OFFSET(F16,-1,))</f>
         <v>4</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="G16" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="36"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
       <c r="L16" s="18"/>
       <c r="M16" s="12"/>
       <c r="N16" s="24"/>
@@ -3121,13 +3134,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F17,-1,))+IF(ISERROR(OFFSET(F17,-1,)*1),0,OFFSET(F17,-1,))</f>
         <v>5</v>
       </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="36"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="33"/>
       <c r="L17" s="18"/>
       <c r="M17" s="12" t="s">
         <v>68</v>
@@ -3160,13 +3173,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F18,-1,))+IF(ISERROR(OFFSET(F18,-1,)*1),0,OFFSET(F18,-1,))</f>
         <v>6</v>
       </c>
-      <c r="G18" s="34" t="s">
+      <c r="G18" s="31" t="s">
         <v>69</v>
       </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="36"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="33"/>
       <c r="L18" s="18"/>
       <c r="M18" s="12" t="s">
         <v>70</v>
@@ -3199,13 +3212,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>7</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="36"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="33"/>
       <c r="L19" s="18"/>
       <c r="M19" s="12"/>
       <c r="N19" s="24"/>
@@ -3236,13 +3249,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>8</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="G20" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="36"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="33"/>
       <c r="L20" s="18"/>
       <c r="M20" s="12" t="s">
         <v>71</v>
@@ -3275,13 +3288,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F21,-1,))+IF(ISERROR(OFFSET(F21,-1,)*1),0,OFFSET(F21,-1,))</f>
         <v>9</v>
       </c>
-      <c r="G21" s="34" t="s">
+      <c r="G21" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="36"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="33"/>
       <c r="L21" s="18"/>
       <c r="M21" s="12" t="s">
         <v>73</v>
@@ -3314,13 +3327,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>10</v>
       </c>
-      <c r="G22" s="34" t="s">
+      <c r="G22" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="36"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="33"/>
       <c r="L22" s="18"/>
       <c r="M22" s="12" t="s">
         <v>75</v>
@@ -3353,13 +3366,13 @@
         <f ca="1">ROW()-ROW(OFFSET(F23,-1,))+IF(ISERROR(OFFSET(F23,-1,)*1),0,OFFSET(F23,-1,))</f>
         <v>11</v>
       </c>
-      <c r="G23" s="34" t="s">
+      <c r="G23" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="36"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="33"/>
       <c r="L23" s="18"/>
       <c r="M23" s="12"/>
       <c r="N23" s="17"/>
@@ -3390,13 +3403,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>12</v>
       </c>
-      <c r="G24" s="34" t="s">
+      <c r="G24" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="36"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="33"/>
       <c r="L24" s="18"/>
       <c r="M24" s="12" t="s">
         <v>77</v>
@@ -3429,13 +3442,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>13</v>
       </c>
-      <c r="G25" s="34" t="s">
+      <c r="G25" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="35"/>
-      <c r="K25" s="36"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="33"/>
       <c r="L25" s="18"/>
       <c r="M25" s="12" t="s">
         <v>79</v>
@@ -3468,13 +3481,13 @@
         <f t="shared" ca="1" si="3"/>
         <v>14</v>
       </c>
-      <c r="G26" s="34" t="s">
+      <c r="G26" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35"/>
-      <c r="K26" s="36"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="33"/>
       <c r="L26" s="18"/>
       <c r="M26" s="12" t="s">
         <v>81</v>
@@ -3507,13 +3520,13 @@
         <f t="shared" ref="F27" ca="1" si="9">ROW()-ROW(OFFSET(F27,-1,))+IF(ISERROR(OFFSET(F27,-1,)*1),0,OFFSET(F27,-1,))</f>
         <v>15</v>
       </c>
-      <c r="G27" s="34" t="s">
+      <c r="G27" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="35"/>
-      <c r="K27" s="36"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="33"/>
       <c r="L27" s="18"/>
       <c r="M27" s="12"/>
       <c r="N27" s="26"/>
@@ -3546,6 +3559,11 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="G27:K27"/>
+    <mergeCell ref="G23:K23"/>
+    <mergeCell ref="G26:K26"/>
+    <mergeCell ref="G24:K24"/>
+    <mergeCell ref="G25:K25"/>
     <mergeCell ref="G13:K13"/>
     <mergeCell ref="G22:K22"/>
     <mergeCell ref="G20:K20"/>
@@ -3559,11 +3577,6 @@
     <mergeCell ref="G18:K18"/>
     <mergeCell ref="G19:K19"/>
     <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G27:K27"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G26:K26"/>
-    <mergeCell ref="G24:K24"/>
-    <mergeCell ref="G25:K25"/>
   </mergeCells>
   <conditionalFormatting sqref="E28">
     <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
@@ -3615,10 +3628,10 @@
       <c r="M1" s="7"/>
     </row>
     <row r="2" spans="2:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
       <c r="J2" s="19"/>
       <c r="K2" s="19" t="s">
         <v>1</v>
@@ -3629,10 +3642,10 @@
       <c r="M2" s="19"/>
     </row>
     <row r="3" spans="2:20" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3">
         <v>0.375</v>
@@ -3736,14 +3749,14 @@
       <c r="E12" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="33"/>
+      <c r="G12" s="37"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="37"/>
+      <c r="K12" s="38"/>
       <c r="L12" s="22" t="s">
         <v>6</v>
       </c>
@@ -3771,13 +3784,13 @@
         <f t="shared" ref="F13:F22" ca="1" si="0">ROW()-ROW(OFFSET(F13,-1,))+IF(ISERROR(OFFSET(F13,-1,)*1),0,OFFSET(F13,-1,))</f>
         <v>1</v>
       </c>
-      <c r="G13" s="34" t="s">
+      <c r="G13" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="36"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="33"/>
       <c r="L13" s="18"/>
       <c r="M13" s="12"/>
       <c r="N13" s="24"/>
@@ -3808,16 +3821,16 @@
         <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
-      <c r="G14" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
-      <c r="J14" s="35"/>
-      <c r="K14" s="36"/>
+      <c r="G14" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="33"/>
       <c r="L14" s="18"/>
       <c r="M14" s="12" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="N14" s="24"/>
       <c r="O14" s="17"/>
@@ -3847,13 +3860,13 @@
         <f t="shared" ca="1" si="0"/>
         <v>3</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="G15" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="36"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="33"/>
       <c r="L15" s="18"/>
       <c r="M15" s="12"/>
       <c r="N15" s="24"/>
@@ -3884,24 +3897,26 @@
         <f t="shared" ca="1" si="0"/>
         <v>4</v>
       </c>
-      <c r="G16" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="36"/>
+      <c r="G16" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="33"/>
       <c r="L16" s="18"/>
       <c r="M16" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="N16" s="26"/>
       <c r="O16" s="17"/>
-      <c r="P16" s="17"/>
-      <c r="Q16" s="17"/>
-      <c r="R16" s="17"/>
-      <c r="S16" s="17"/>
-      <c r="T16" s="17"/>
+      <c r="P16" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q16" s="29"/>
+      <c r="R16" s="29"/>
+      <c r="S16" s="29"/>
+      <c r="T16" s="30"/>
     </row>
     <row r="17" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B17" s="9">
@@ -3914,33 +3929,33 @@
       </c>
       <c r="D17" s="10">
         <f t="shared" ca="1" si="3"/>
-        <v>0.49305555555555552</v>
+        <v>0.47916666666666663</v>
       </c>
       <c r="E17" s="11">
-        <v>2.0833333333333332E-2</v>
+        <v>6.9444444444444441E-3</v>
       </c>
       <c r="F17" s="12">
         <f t="shared" ca="1" si="0"/>
         <v>5</v>
       </c>
-      <c r="G17" s="34" t="s">
-        <v>87</v>
-      </c>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
-      <c r="J17" s="35"/>
-      <c r="K17" s="36"/>
+      <c r="G17" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="33"/>
       <c r="L17" s="18"/>
-      <c r="M17" s="12" t="s">
-        <v>86</v>
-      </c>
+      <c r="M17" s="12"/>
       <c r="N17" s="17"/>
       <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
+      <c r="P17" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q17" s="29"/>
+      <c r="R17" s="29"/>
+      <c r="S17" s="29"/>
+      <c r="T17" s="30"/>
     </row>
     <row r="18" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B18" s="9">
@@ -3949,35 +3964,39 @@
       </c>
       <c r="C18" s="10">
         <f ca="1">IF(E18="Select","",IF(AND(F18=1,E18&lt;&gt;"Select"),$K$3,OFFSET(C18,-1,1)))</f>
-        <v>0.49305555555555552</v>
+        <v>0.47916666666666663</v>
       </c>
       <c r="D18" s="10">
         <f ca="1">IF(ISERROR(E18+C18),"",E18+C18)</f>
-        <v>0.53472222222222221</v>
+        <v>0.49999999999999994</v>
       </c>
       <c r="E18" s="11">
-        <v>4.1666666666666664E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="F18" s="12">
         <f ca="1">ROW()-ROW(OFFSET(F18,-1,))+IF(ISERROR(OFFSET(F18,-1,)*1),0,OFFSET(F18,-1,))</f>
         <v>6</v>
       </c>
-      <c r="G18" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="36"/>
+      <c r="G18" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="33"/>
       <c r="L18" s="18"/>
-      <c r="M18" s="12"/>
+      <c r="M18" s="12" t="s">
+        <v>84</v>
+      </c>
       <c r="N18" s="17"/>
       <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="17"/>
+      <c r="P18" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q18" s="29"/>
+      <c r="R18" s="29"/>
+      <c r="S18" s="29"/>
+      <c r="T18" s="30"/>
     </row>
     <row r="19" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="9">
@@ -3986,37 +4005,39 @@
       </c>
       <c r="C19" s="10">
         <f ca="1">IF(E19="Select","",IF(AND(F19=1,E19&lt;&gt;"Select"),$K$3,OFFSET(C19,-1,1)))</f>
-        <v>0.53472222222222221</v>
+        <v>0.49999999999999994</v>
       </c>
       <c r="D19" s="10">
         <f ca="1">IF(ISERROR(E19+C19),"",E19+C19)</f>
-        <v>0.55555555555555558</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="E19" s="11">
-        <v>2.0833333333333332E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="F19" s="12">
         <f ca="1">ROW()-ROW(OFFSET(F19,-1,))+IF(ISERROR(OFFSET(F19,-1,)*1),0,OFFSET(F19,-1,))</f>
         <v>7</v>
       </c>
-      <c r="G19" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="36"/>
+      <c r="G19" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="33"/>
       <c r="L19" s="18"/>
       <c r="M19" s="12" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="N19" s="24"/>
       <c r="O19" s="20"/>
-      <c r="P19" s="20"/>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="17"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="17"/>
+      <c r="P19" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q19" s="29"/>
+      <c r="R19" s="29"/>
+      <c r="S19" s="29"/>
+      <c r="T19" s="30"/>
     </row>
     <row r="20" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="9">
@@ -4025,37 +4046,39 @@
       </c>
       <c r="C20" s="10">
         <f ca="1">IF(E20="Select","",IF(AND(F20=1,E20&lt;&gt;"Select"),$K$3,OFFSET(C20,-1,1)))</f>
-        <v>0.55555555555555558</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="D20" s="10">
         <f ca="1">IF(ISERROR(E20+C20),"",E20+C20)</f>
-        <v>0.58333333333333337</v>
+        <v>0.5625</v>
       </c>
       <c r="E20" s="11">
-        <v>2.7777777777777776E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="F20" s="12">
         <f ca="1">ROW()-ROW(OFFSET(F20,-1,))+IF(ISERROR(OFFSET(F20,-1,)*1),0,OFFSET(F20,-1,))</f>
         <v>8</v>
       </c>
-      <c r="G20" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="36"/>
+      <c r="G20" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="33"/>
       <c r="L20" s="18"/>
       <c r="M20" s="12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="N20" s="24"/>
       <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="17"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="17"/>
+      <c r="P20" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="29"/>
+      <c r="S20" s="29"/>
+      <c r="T20" s="30"/>
     </row>
     <row r="21" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="9">
@@ -4064,37 +4087,39 @@
       </c>
       <c r="C21" s="10">
         <f t="shared" ca="1" si="2"/>
-        <v>0.58333333333333337</v>
+        <v>0.5625</v>
       </c>
       <c r="D21" s="10">
         <f t="shared" ca="1" si="3"/>
-        <v>0.625</v>
+        <v>0.57638888888888884</v>
       </c>
       <c r="E21" s="11">
-        <v>4.1666666666666664E-2</v>
+        <v>1.3888888888888888E-2</v>
       </c>
       <c r="F21" s="12">
         <f t="shared" ca="1" si="0"/>
         <v>9</v>
       </c>
-      <c r="G21" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="36"/>
+      <c r="G21" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="33"/>
       <c r="L21" s="18"/>
       <c r="M21" s="12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="N21" s="24"/>
       <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="17"/>
+      <c r="P21" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q21" s="29"/>
+      <c r="R21" s="29"/>
+      <c r="S21" s="29"/>
+      <c r="T21" s="30"/>
     </row>
     <row r="22" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="9">
@@ -4103,11 +4128,11 @@
       </c>
       <c r="C22" s="10">
         <f t="shared" ref="C22" ca="1" si="5">IF(E22="Select","",IF(AND(F22=1,E22&lt;&gt;"Select"),$K$3,OFFSET(C22,-1,1)))</f>
-        <v>0.625</v>
+        <v>0.57638888888888884</v>
       </c>
       <c r="D22" s="10">
         <f t="shared" ref="D22" ca="1" si="6">IF(ISERROR(E22+C22),"",E22+C22)</f>
-        <v>0.63194444444444442</v>
+        <v>0.58333333333333326</v>
       </c>
       <c r="E22" s="11">
         <v>6.9444444444444441E-3</v>
@@ -4116,22 +4141,24 @@
         <f t="shared" ca="1" si="0"/>
         <v>10</v>
       </c>
-      <c r="G22" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="36"/>
+      <c r="G22" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="33"/>
       <c r="L22" s="18"/>
       <c r="M22" s="12"/>
       <c r="N22" s="24"/>
       <c r="O22" s="17"/>
-      <c r="P22" s="17"/>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="17"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="17"/>
+      <c r="P22" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q22" s="29"/>
+      <c r="R22" s="29"/>
+      <c r="S22" s="29"/>
+      <c r="T22" s="30"/>
     </row>
     <row r="23" spans="2:20" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B23" s="9">
@@ -4140,11 +4167,11 @@
       </c>
       <c r="C23" s="10">
         <f t="shared" ref="C23:C26" ca="1" si="7">IF(E23="Select","",IF(AND(F23=1,E23&lt;&gt;"Select"),$K$3,OFFSET(C23,-1,1)))</f>
-        <v>0.63194444444444442</v>
+        <v>0.58333333333333326</v>
       </c>
       <c r="D23" s="10">
         <f t="shared" ref="D23:D26" ca="1" si="8">IF(ISERROR(E23+C23),"",E23+C23)</f>
-        <v>0.63888888888888884</v>
+        <v>0.59027777777777768</v>
       </c>
       <c r="E23" s="11">
         <v>6.9444444444444441E-3</v>
@@ -4153,13 +4180,13 @@
         <f t="shared" ref="F23:F26" ca="1" si="9">ROW()-ROW(OFFSET(F23,-1,))+IF(ISERROR(OFFSET(F23,-1,)*1),0,OFFSET(F23,-1,))</f>
         <v>11</v>
       </c>
-      <c r="G23" s="34" t="s">
-        <v>94</v>
-      </c>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="36"/>
+      <c r="G23" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="33"/>
       <c r="L23" s="18"/>
       <c r="M23" s="12"/>
       <c r="N23" s="17"/>
@@ -4177,11 +4204,11 @@
       </c>
       <c r="C24" s="10">
         <f t="shared" ca="1" si="7"/>
-        <v>0.63888888888888884</v>
+        <v>0.59027777777777768</v>
       </c>
       <c r="D24" s="10">
         <f t="shared" ca="1" si="8"/>
-        <v>0.64583333333333326</v>
+        <v>0.5972222222222221</v>
       </c>
       <c r="E24" s="11">
         <v>6.9444444444444441E-3</v>
@@ -4190,13 +4217,13 @@
         <f t="shared" ca="1" si="9"/>
         <v>12</v>
       </c>
-      <c r="G24" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
-      <c r="K24" s="36"/>
+      <c r="G24" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="33"/>
       <c r="L24" s="18"/>
       <c r="M24" s="12"/>
       <c r="N24" s="17"/>
@@ -4214,26 +4241,26 @@
       </c>
       <c r="C25" s="10">
         <f t="shared" ca="1" si="7"/>
-        <v>0.64583333333333326</v>
+        <v>0.5972222222222221</v>
       </c>
       <c r="D25" s="10">
         <f t="shared" ca="1" si="8"/>
-        <v>0.68749999999999989</v>
-      </c>
-      <c r="E25" s="11">
-        <v>4.1666666666666664E-2</v>
+        <v>0.70138888888888873</v>
+      </c>
+      <c r="E25" s="39">
+        <v>0.10416666666666667</v>
       </c>
       <c r="F25" s="12">
         <f t="shared" ca="1" si="9"/>
         <v>13</v>
       </c>
-      <c r="G25" s="34" t="s">
-        <v>92</v>
-      </c>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="35"/>
-      <c r="K25" s="36"/>
+      <c r="G25" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="33"/>
       <c r="L25" s="18"/>
       <c r="M25" s="12"/>
       <c r="N25" s="24"/>
@@ -4251,26 +4278,26 @@
       </c>
       <c r="C26" s="10">
         <f t="shared" ca="1" si="7"/>
-        <v>0.68749999999999989</v>
+        <v>0.70138888888888873</v>
       </c>
       <c r="D26" s="10">
         <f t="shared" ca="1" si="8"/>
-        <v>0.70833333333333326</v>
+        <v>0.70138888888888873</v>
       </c>
       <c r="E26" s="11">
-        <v>2.0833333333333332E-2</v>
+        <v>0</v>
       </c>
       <c r="F26" s="12">
         <f t="shared" ca="1" si="9"/>
         <v>14</v>
       </c>
-      <c r="G26" s="34" t="s">
+      <c r="G26" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35"/>
-      <c r="K26" s="36"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="33"/>
       <c r="L26" s="18"/>
       <c r="M26" s="12"/>
       <c r="N26" s="24"/>
@@ -4284,10 +4311,10 @@
     <row r="27" spans="2:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E27" s="13">
         <f>SUM(E13:E26)</f>
-        <v>0.33333333333333326</v>
-      </c>
-    </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.2">
+        <v>0.3263888888888889</v>
+      </c>
+    </row>
+    <row r="30" spans="2:20" ht="16" x14ac:dyDescent="0.2">
       <c r="B30" s="8" t="s">
         <v>10</v>
       </c>
@@ -4303,6 +4330,8 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G23:K23"/>
     <mergeCell ref="G26:K26"/>
     <mergeCell ref="F2:I2"/>
     <mergeCell ref="F3:I3"/>
@@ -4312,24 +4341,25 @@
     <mergeCell ref="G15:K15"/>
     <mergeCell ref="G14:K14"/>
     <mergeCell ref="G19:K19"/>
+    <mergeCell ref="G20:K20"/>
     <mergeCell ref="G21:K21"/>
-    <mergeCell ref="G22:K22"/>
     <mergeCell ref="G24:K24"/>
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="G18:K18"/>
-    <mergeCell ref="G20:K20"/>
-    <mergeCell ref="G23:K23"/>
-    <mergeCell ref="G25:K25"/>
+    <mergeCell ref="G22:K22"/>
   </mergeCells>
   <conditionalFormatting sqref="E27">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>#REF!&lt;&gt;#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter time as H:MM:SS (update AM/PM as necessary)." sqref="K3:L11" xr:uid="{90388A18-C8F8-4289-9C54-D45BB899292C}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E13:E26" xr:uid="{442B30E4-E34A-4905-A5CF-6B3CFE36CE25}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E13:E24 E26" xr:uid="{442B30E4-E34A-4905-A5CF-6B3CFE36CE25}">
       <formula1>"0:00, 0:05, 0:10, 0:15, 0:20, 0:25, 0:30, 0:35, 0:40, 0:45, 0:50, 0:55, 1:00, 1:15, 1:30"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E25" xr:uid="{8F7D9711-0EFA-2740-9F5F-40739E0BC102}">
+      <formula1>"0:00, 0:05, 0:10, 0:15, 0:20, 0:25, 0:30, 0:35, 0:40, 0:45, 0:50, 0:55, 1:00, 1:15, 1:30, 2:30"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>